<commit_message>
Fix: Personalização de variáveis e planilha modelo
</commit_message>
<xml_diff>
--- a/uploads/contatos_sigma_pdv_v2.xlsx
+++ b/uploads/contatos_sigma_pdv_v2.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Contatos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contatos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -426,7 +426,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -486,14 +486,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ENVIADO</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>14/04/2026 16:21</t>
-        </is>
-      </c>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -516,6 +513,8 @@
           <t>PENDENTE</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>